<commit_message>
feat(draft): drop the Kraj (country) column from the data model
Country is no longer imported or used. Remove it everywhere:
- Player/PlayerWithManager/DraftPoolImport types
- import parser + generated template (now 4 cols: Imię i Nazwisko, Liga,
  Klub, Pozycja) and both import pages' instructions
- draft snapshot + add-player API (no longer select/insert country)
- draft UI: Kraj filter, table column, and add-player field
- seed/template scripts (also drop Goalkeeper from seed positions)
- migration 023 drops players.country (idempotent)

Code no longer references the column, so it works whether or not 023 has
been applied yet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/migrations/player-import-template.xlsx
+++ b/migrations/player-import-template.xlsx
@@ -397,13 +397,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="26"/>
-    <col min="2" max="2" customWidth="1" width="16"/>
+    <col min="2" max="2" customWidth="1" width="20"/>
     <col min="3" max="3" customWidth="1" width="20"/>
-    <col min="4" max="4" customWidth="1" width="20"/>
-    <col min="5" max="5" customWidth="1" width="14"/>
+    <col min="4" max="4" customWidth="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -411,15 +410,12 @@
         <v>Imię i Nazwisko</v>
       </c>
       <c r="B1" t="str">
-        <v>Kraj</v>
+        <v>Liga</v>
       </c>
       <c r="C1" t="str">
-        <v>Liga</v>
+        <v>Klub</v>
       </c>
       <c r="D1" t="str">
-        <v>Klub</v>
-      </c>
-      <c r="E1" t="str">
         <v>Pozycja</v>
       </c>
     </row>
@@ -428,15 +424,12 @@
         <v>Lionel Messi</v>
       </c>
       <c r="B2" t="str">
-        <v>Argentyna</v>
+        <v>MLS</v>
       </c>
       <c r="C2" t="str">
-        <v>MLS</v>
+        <v>Inter Miami</v>
       </c>
       <c r="D2" t="str">
-        <v>Inter Miami</v>
-      </c>
-      <c r="E2" t="str">
         <v>Napastnik</v>
       </c>
     </row>
@@ -445,15 +438,12 @@
         <v>Virgil van Dijk</v>
       </c>
       <c r="B3" t="str">
-        <v>Holandia</v>
+        <v>Premier League</v>
       </c>
       <c r="C3" t="str">
-        <v>Premier League</v>
+        <v>Liverpool FC</v>
       </c>
       <c r="D3" t="str">
-        <v>Liverpool FC</v>
-      </c>
-      <c r="E3" t="str">
         <v>Obrońca</v>
       </c>
     </row>
@@ -462,15 +452,12 @@
         <v>Luka Modrić</v>
       </c>
       <c r="B4" t="str">
-        <v>Chorwacja</v>
+        <v>La Liga</v>
       </c>
       <c r="C4" t="str">
-        <v>La Liga</v>
+        <v>Real Madrid</v>
       </c>
       <c r="D4" t="str">
-        <v>Real Madrid</v>
-      </c>
-      <c r="E4" t="str">
         <v>Pomocnik</v>
       </c>
     </row>
@@ -479,21 +466,18 @@
         <v>Robert Lewandowski</v>
       </c>
       <c r="B5" t="str">
-        <v>Polska</v>
+        <v>La Liga</v>
       </c>
       <c r="C5" t="str">
-        <v>La Liga</v>
+        <v>FC Barcelona</v>
       </c>
       <c r="D5" t="str">
-        <v>FC Barcelona</v>
-      </c>
-      <c r="E5" t="str">
         <v>Napastnik</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>